<commit_message>
Update analysis Excel files across multiple departments
- Modified Betygsrapportering.xlsx, Betygsskalor.xlsx, Bloom-taxonomi.xlsx, Examinationsformer.xlsx, Frasningskonsistens.xlsx, Färkunskapskrav.xlsx, Introfras.xlsx, Nedlagda kursreferenser.xlsx, Omfång på lärandemål.xlsx, Programkurser olänkade.xlsx, Samstämmighet svenska och engelska.xlsx, Stavfel och språkbruk.xlsx, and Övrigt.xlsx in the 01 IIT, 02 IHV, 03 IKS, and 04 ISLL directories.
- Adjusted links and content in Programkurser olänkade.md for accuracy.
- Ensured all changes reflect the latest data and formatting requirements.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/03 IKS/Analys/Programkurser olänkade.xlsx
+++ b/vault-dalarna-university/03 IKS/Analys/Programkurser olänkade.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Programkurser olänkade" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$115</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E116"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2794,7 +2794,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>SMHTA</t>
+          <t>SMINA</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2804,17 +2804,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Bullet beskriver val mellan flera kurser</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>`Eller Examensarbete för Magisterexamen i Turismvetenskap` (15 hp); rad: - Eller Examensarbete för Magisterexamen i Turismvetenskap, 15 hp</t>
+          <t>`Avancerad mikroteori` (7,5 hp); rad: - Avancerad mikroteori, 7,5 hp</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SMHTA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SMINA</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2836,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>`Avancerad mikroteori` (7,5 hp); rad: - Avancerad mikroteori, 7,5 hp</t>
+          <t>`Samhällsekonomisk utvärdering av offentliga projekt` (7,5 hp); rad: - Samhällsekonomisk utvärdering av offentliga projekt, 7,5 hp</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -2848,7 +2848,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>SMINA</t>
+          <t>SPARG</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2863,12 +2863,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>`Samhällsekonomisk utvärdering av offentliga projekt` (7,5 hp); rad: - Samhällsekonomisk utvärdering av offentliga projekt, 7,5 hp</t>
+          <t>`Arbetsrätt i personalarbetets praktik` (15 hp); rad: - Arbetsrätt i personalarbetets praktik, 15 hp</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SMINA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>`Arbetsrätt i personalarbetets praktik` (15 hp); rad: - Arbetsrätt i personalarbetets praktik, 15 hp</t>
+          <t>`Grunder i personalekonomisk styrning` (15 hp); rad: - Grunder i personalekonomisk styrning, 15 hp</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>`Grunder i personalekonomisk styrning` (15 hp); rad: - Grunder i personalekonomisk styrning, 15 hp</t>
+          <t>`Personalarbete med praktik` (15 hp); rad: - Personalarbete med praktik, 15 hp</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>`Personalarbete med praktik` (15 hp); rad: - Personalarbete med praktik, 15 hp</t>
+          <t>`Arbetsmarknad i ett jämförande internationellt perspektiv` (7,5 hp); rad: - Arbetsmarknad i ett jämförande internationellt perspektiv, 7,5 hp</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>`Arbetsmarknad i ett jämförande internationellt perspektiv` (7,5 hp); rad: - Arbetsmarknad i ett jämförande internationellt perspektiv, 7,5 hp</t>
+          <t>`Arbetsmiljökunskap i ett jämförande internationellt perspektiv` (7,5 hp); rad: - Arbetsmiljökunskap i ett jämförande internationellt perspektiv, 7,5 hp</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2998,7 +2998,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>`Arbetsmiljökunskap i ett jämförande internationellt perspektiv` (7,5 hp); rad: - Arbetsmiljökunskap i ett jämförande internationellt perspektiv, 7,5 hp</t>
+          <t>`Examensarbete inom arbetsvetenskap` (15 hp); rad: - Examensarbete inom arbetsvetenskap, 15 hp</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -3025,7 +3025,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>`Examensarbete inom arbetsvetenskap` (15 hp); rad: - Examensarbete inom arbetsvetenskap, 15 hp</t>
+          <t>`Forskningsprocess och analysmetoder` (7,5 hp); rad: - Forskningsprocess och analysmetoder, 7,5 hp</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>`Forskningsprocess och analysmetoder` (7,5 hp); rad: - Forskningsprocess och analysmetoder, 7,5 hp</t>
+          <t>`Komplexa arbetsorganisationer` (7,5 hp); rad: - Komplexa arbetsorganisationer, 7,5 hp</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>`Komplexa arbetsorganisationer` (7,5 hp); rad: - Komplexa arbetsorganisationer, 7,5 hp</t>
+          <t>`Komplexa sociala processer i arbetslivet` (7,5 hp); rad: - Komplexa sociala processer i arbetslivet, 7,5 hp</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>`Komplexa sociala processer i arbetslivet` (7,5 hp); rad: - Komplexa sociala processer i arbetslivet, 7,5 hp</t>
+          <t>`Vetenskap och metod` (7,5 hp); rad: - Vetenskap och metod, 7,5 hp</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -3118,7 +3118,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>SPARG</t>
+          <t>SSHVG</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3133,12 +3133,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>`Vetenskap och metod` (7,5 hp); rad: - Vetenskap och metod, 7,5 hp</t>
+          <t>`Inriktning sociologi II` (30 hp); rad: - Inriktning sociologi II, 30 hp</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>`Inriktning sociologi II` (30 hp); rad: - Inriktning sociologi II, 30 hp</t>
+          <t>`Examensarbete för högskoleexamen i Sociologi` (7,5 hp); rad: - Examensarbete för högskoleexamen i Sociologi, 7,5 hp</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>`Examensarbete för högskoleexamen i Sociologi` (7,5 hp); rad: - Examensarbete för högskoleexamen i Sociologi, 7,5 hp</t>
+          <t>`Makt och samhälle` (7,5 hp); rad: - Makt och samhälle, 7,5 hp</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>`Makt och samhälle` (7,5 hp); rad: - Makt och samhälle, 7,5 hp</t>
+          <t>`Samhällsvetenskapliga metoder I` (7,5 hp); rad: - Samhällsvetenskapliga metoder I, 7,5 hp</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>`Samhällsvetenskapliga metoder I` (7,5 hp); rad: - Samhällsvetenskapliga metoder I, 7,5 hp</t>
+          <t>`Inriktning statsvetenskap II` (30 hp); rad: - Inriktning statsvetenskap II, 30 hp</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -3268,7 +3268,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>`Inriktning statsvetenskap II` (30 hp); rad: - Inriktning statsvetenskap II, 30 hp</t>
+          <t>`Inriktning sociologi III` (30 hp); rad: - Inriktning sociologi III, 30 hp</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>`Inriktning sociologi III` (30 hp); rad: - Inriktning sociologi III, 30 hp</t>
+          <t>`Examensarbete för kandidatexamen i sociologi` (15 hp); rad: - Examensarbete för kandidatexamen i sociologi, 15 hp</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -3322,7 +3322,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>`Examensarbete för kandidatexamen i sociologi` (15 hp); rad: - Examensarbete för kandidatexamen i sociologi, 15 hp</t>
+          <t>`Fördjupningskurs i sociologisk teori` (7,5 hp); rad: - Fördjupningskurs i sociologisk teori, 7,5 hp</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -3349,7 +3349,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>`Fördjupningskurs i sociologisk teori` (7,5 hp); rad: - Fördjupningskurs i sociologisk teori, 7,5 hp</t>
+          <t>`Samhällsvetenskapliga metoder II` (7,5 hp); rad: - Samhällsvetenskapliga metoder II, 7,5 hp</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>`Samhällsvetenskapliga metoder II` (7,5 hp); rad: - Samhällsvetenskapliga metoder II, 7,5 hp</t>
+          <t>`Inriktning statsvetenskap III` (30 hp); rad: - Inriktning statsvetenskap III, 30 hp</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
@@ -3403,7 +3403,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>`Inriktning statsvetenskap III` (30 hp); rad: - Inriktning statsvetenskap III, 30 hp</t>
+          <t>`Samhällsvetenskapliga metoder II inriktning statsvetenskap` (7,5 hp); rad: - Samhällsvetenskapliga metoder II inriktning statsvetenskap, 7,5 hp</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -3425,12 +3425,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Kursraden ser avbruten/feltrycklig ut</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>`Samhällsvetenskapliga metoder II inriktning statsvetenskap` (7,5 hp); rad: - Samhällsvetenskapliga metoder II inriktning statsvetenskap, 7,5 hp</t>
+          <t>`Valbar termin (med möjlighet till internationellt utbyte eller läsning av valfri temakurs/kurser om` (30 hp); rad: - Valbar termin (med möjlighet till internationellt utbyte eller läsning av valfri temakurs/kurser om, 30 hp</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
@@ -3452,12 +3452,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Kursraden ser avbruten/feltrycklig ut</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>`Valbar termin (med möjlighet till internationellt utbyte eller läsning av valfri temakurs/kurser om` (30 hp); rad: - Valbar termin (med möjlighet till internationellt utbyte eller läsning av valfri temakurs/kurser om, 30 hp</t>
+          <t>Programtext `Samhällsvetenskapliga metoder I – inriktning statsvetenskap` ≠ kursplanens namn `Samhällsvetenskapliga metoder I - inriktning statsvetenskap` (kurskod `GSK2PT`); rad: - [[GSK2PT|Samhällsvetenskapliga metoder I – inriktning statsvetenskap]], 7,5 hp</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -3469,7 +3469,7 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>SSHVG</t>
+          <t>STMGG</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -3479,17 +3479,17 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Programtext `Samhällsvetenskapliga metoder I – inriktning statsvetenskap` ≠ kursplanens namn `Samhällsvetenskapliga metoder I - inriktning statsvetenskap` (kurskod `GSK2PT`); rad: - [[GSK2PT|Samhällsvetenskapliga metoder I – inriktning statsvetenskap]], 7,5 hp</t>
+          <t>`Festival och Event Management` (7,5 hp); rad: - Festival och Event Management, 7,5 hp</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=STMGG</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>`Festival och Event Management` (7,5 hp); rad: - Festival och Event Management, 7,5 hp</t>
+          <t>`Turismstudier utomlands` (30 hp); rad: - Turismstudier utomlands, 30 hp</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -3538,7 +3538,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>`Turismstudier utomlands` (30 hp); rad: - Turismstudier utomlands, 30 hp</t>
+          <t>`Kvantitativa forskningsmetoder` (7,5 hp); rad: - Kvantitativa forskningsmetoder, 7,5 hp</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
@@ -3547,35 +3547,8 @@
         </is>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>STMGG</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>`Kvantitativa forskningsmetoder` (7,5 hp); rad: - Kvantitativa forskningsmetoder, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E116" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=STMGG</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E116"/>
+  <autoFilter ref="A1:E115"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -3805,8 +3778,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId226"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A115" r:id="rId227"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A116" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E116" r:id="rId230"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analysis files for Dalarna University programs
- Modified multiple Excel files in the "03 IKS" and "04 ISLL" directories, including:
  - Programkurser olänkade.xlsx
  - Samstämmighet svenska och engelska.xlsx
  - Stavfel och språkbruk.xlsx
  - Övrigt.xlsx
  - Betygsrapportering.xlsx
  - Betygsskalor.xlsx
  - Bloom-taxonomi.xlsx
  - Examinationsformer.xlsx
  - Frasningskonsistens.xlsx
  - Förkunskapskrav.xlsx
  - Introfras.xlsx
  - Nedlagda kursreferenser.xlsx
  - Omfång på lärandemål.xlsx
- Updated markdown file for Programkurser olänkade with corrected download links and updated findings count.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/03 IKS/Analys/Programkurser olänkade.xlsx
+++ b/vault-dalarna-university/03 IKS/Analys/Programkurser olänkade.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Programkurser olänkade" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olänkade'!$A$1:$E$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -823,7 +823,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>HAFSA</t>
+          <t>KFTPG</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -833,24 +833,24 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Programtext `Afrikanska samhällen i förändring` ≠ kursplanens namn `Afrikanska studier: Afrikanska samhällen i förändring` (kurskod `AS3022`); rad: - [[AS3022|Afrikanska samhällen i förändring]], 12 hp</t>
+          <t>`Digitalefterbearbetning av ljud och bild` (15 hp); rad: - Digitalefterbearbetning av ljud och bild, 15 hp</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=HAFSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KFTPG</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>HAFSA</t>
+          <t>KLJMG</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -860,24 +860,24 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Programtext `Religion och politik i afrikanska samhällen` ≠ kursplanens namn `Afrikanska studier: Religion och politik i afrikanska samhällen` (kurskod `AS3023`); rad: - [[AS3023|Religion och politik i afrikanska samhällen]], 9 hp</t>
+          <t>`Konceptutveckling inom medieproduktion i Ljud- och musikproduktion` (7,5 hp); rad: - Konceptutveckling inom medieproduktion i Ljud- och musikproduktion, 7,5 hp</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=HAFSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>HAFSA</t>
+          <t>KLJMG</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -887,24 +887,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Programtext `Utbildning och förändring i afrikanska samhällen` ≠ kursplanens namn `Afrikanska studier: Utbildning och förändring i afrikanska samhällen` (kurskod `AS3021`); rad: - [[AS3021|Utbildning och förändring i afrikanska samhällen]], 8 hp</t>
+          <t>`Arbetsplatsförlagd utbildning för medieproduktion` (15 hp); rad: - Arbetsplatsförlagd utbildning för medieproduktion, 15 hp</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=HAFSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>HAFSA</t>
+          <t>KLJMG</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Programtext `Litteratur och politik i det samtida Afrika` ≠ kursplanens namn `Afrikanska studier: Litteratur och politik i det samtida Afrika` (kurskod `AS3017`); rad: - [[AS3017|Litteratur och politik i det samtida Afrika]], 7 hp</t>
+          <t>Programtext `Produktionsprocesser och -villkor inom musikproduktion` ≠ kursplanens namn `Produktionsprocesser och - villkor inom musikproduktion` (kurskod `LP1072`); rad: - [[LP1072|Produktionsprocesser och -villkor inom musikproduktion]], 7,5 hp</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=HAFSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>HAFSA</t>
+          <t>KMLJG</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -941,24 +941,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Programtext `Ekonomisk utveckling i Afrika, en introduktion` ≠ kursplanens namn `Afrikanska studier: Ekonomisk utveckling i Afrika, en introduktion` (kurskod `AS3019`); rad: - [[AS3019|Ekonomisk utveckling i Afrika, en introduktion]], 7 hp</t>
+          <t>`Audioteknologi I` (7,5 hp); rad: - Audioteknologi I, 7,5 hp</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=HAFSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>HAFSA</t>
+          <t>KMLJG</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -968,24 +968,24 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Programtext `Internationell hälsa med fokus på nutrition i ett genus- och ekonomiskt perspektiv` ≠ kursplanens namn `Afrikanska studier: Internationell hälsa med fokus på nutrition i ett genus- och ekonomiskt perspektiv` (kurskod `AS3014`); rad: - [[AS3014|Internationell hälsa med fokus på nutrition i ett genus- och ekonomiskt perspektiv]], 7hp</t>
+          <t>`Audioteknologi II` (7,5 hp); rad: - Audioteknologi II, 7,5 hp</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=HAFSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>HAFSA</t>
+          <t>KMLJG</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -995,24 +995,24 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Programtext `Det urbana rummet och urbaniseringspolitik i Afrika söder om Sahara` ≠ kursplanens namn `Afrikanska studier: Det urbana rummet och urbaniseringspolitik i Afrika söder om Sahara` (kurskod `AS3018`); rad: - [[AS3018|Det urbana rummet och urbaniseringspolitik i Afrika söder om Sahara]], 7 hp</t>
+          <t>`Introduktion till Musik- och ljuddesign` (7,5 hp); rad: - Introduktion till Musik- och ljuddesign, 7,5 hp</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=HAFSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>KFTPG</t>
+          <t>KMLJG</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1027,19 +1027,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>`Digitalefterbearbetning av ljud och bild` (15 hp); rad: - Digitalefterbearbetning av ljud och bild, 15 hp</t>
+          <t>`Ljudskapande och ljudsyntes` (7,5 hp); rad: - Ljudskapande och ljudsyntes, 7,5 hp</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KFTPG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>KLJMG</t>
+          <t>KMLJG</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1054,19 +1054,19 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>`Konceptutveckling inom medieproduktion i Ljud- och musikproduktion` (7,5 hp); rad: - Konceptutveckling inom medieproduktion i Ljud- och musikproduktion, 7,5 hp</t>
+          <t>`Vår tids musik och musikliv` (7,5 hp); rad: - Vår tids musik och musikliv, 7,5 hp</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>KLJMG</t>
+          <t>KMLJG</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1081,19 +1081,19 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>`Arbetsplatsförlagd utbildning för medieproduktion` (15 hp); rad: - Arbetsplatsförlagd utbildning för medieproduktion, 15 hp</t>
+          <t>`Företagsekonomi för musikbranschen` (7,5 hp); rad: - Företagsekonomi för musikbranschen, 7,5 hp</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>KLJMG</t>
+          <t>KMLJG</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1103,24 +1103,24 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Programtext `Produktionsprocesser och -villkor inom musikproduktion` ≠ kursplanens namn `Produktionsprocesser och - villkor inom musikproduktion` (kurskod `LP1072`); rad: - [[LP1072|Produktionsprocesser och -villkor inom musikproduktion]], 7,5 hp</t>
+          <t>`Musikbranschen` (7,5 hp); rad: - Musikbranschen, 7,5 hp</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KLJMG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>KMLJG</t>
+          <t>L7I9A</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1135,19 +1135,19 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>`Audioteknologi I` (7,5 hp); rad: - Audioteknologi I, 7,5 hp</t>
+          <t>`Sociala relationer, konflikter och makt för ämneslärare årskurs 7–9 - AIL` (7,5 hp); rad: - Sociala relationer, konflikter och makt för ämneslärare årskurs 7–9 - AIL, 7,5 hp</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=L7I9A</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>KMLJG</t>
+          <t>L7I9A</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1162,19 +1162,19 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>`Audioteknologi II` (7,5 hp); rad: - Audioteknologi II, 7,5 hp</t>
+          <t>`Utvärdering och utvecklingsarbete för ämneslärare årskurs 7–9 – AIL` (7,5 hp); rad: - Utvärdering och utvecklingsarbete för ämneslärare årskurs 7–9 – AIL, 7,5 hp</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=L7I9A</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>KMLJG</t>
+          <t>L7I9A</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1189,19 +1189,19 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>`Introduktion till Musik- och ljuddesign` (7,5 hp); rad: - Introduktion till Musik- och ljuddesign, 7,5 hp</t>
+          <t>`Verksamhetsförlagd utbildning 3 för ämneslärare årskurs 7–9 - AIL` (15 hp); rad: - Verksamhetsförlagd utbildning 3 för ämneslärare årskurs 7–9 - AIL, 15 hp</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=L7I9A</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>KMLJG</t>
+          <t>L7I9A</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1216,19 +1216,19 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>`Ljudskapande och ljudsyntes` (7,5 hp); rad: - Ljudskapande och ljudsyntes, 7,5 hp</t>
+          <t>`Vetenskapsteori och utbildningsvetenskaplig forskning för ämneslärare årskurs 7–9 - AIL` (7,5 hp); rad: - Vetenskapsteori och utbildningsvetenskaplig forskning för ämneslärare årskurs 7–9 - AIL, 7,5 hp</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=L7I9A</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>KMLJG</t>
+          <t>L7I9A</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1243,19 +1243,19 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>`Vår tids musik och musikliv` (7,5 hp); rad: - Vår tids musik och musikliv, 7,5 hp</t>
+          <t>`_Examensarbete i matematik för ämneslärarexamen inriktning grundskolans årskurs 7–9` (15 hp); rad: - _Examensarbete i matematik för ämneslärarexamen inriktning grundskolans årskurs 7–9, 15 hp</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=L7I9A</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>KMLJG</t>
+          <t>LBF3A</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1270,19 +1270,19 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>`Företagsekonomi för musikbranschen` (7,5 hp); rad: - Företagsekonomi för musikbranschen, 7,5 hp</t>
+          <t>`Didaktik och ledarskap i förskoleklass och grundskolans åk 1–3` (15 hp); rad: - Didaktik och ledarskap i förskoleklass och grundskolans åk 1–3, 15 hp</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>KMLJG</t>
+          <t>LBF3A</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1297,19 +1297,19 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>`Musikbranschen` (7,5 hp); rad: - Musikbranschen, 7,5 hp</t>
+          <t>`Utvärdering och utvecklingsarbete i förskoleklass och grundskolans åk 1–3` (15 hp); rad: - Utvärdering och utvecklingsarbete i förskoleklass och grundskolans åk 1–3, 15 hp</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>KMLJG</t>
+          <t>LBF3A</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1324,19 +1324,19 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Programtext `Examensarbete för högskoleexamen i musik­ och ljuddesign` ≠ kursplanens namn `Examensarbete för högskoleexamen i musik- och ljuddesign` (kurskod `LP1032`); rad: - [[LP1032|Examensarbete för högskoleexamen i musik­ och ljuddesign]], 15 hp</t>
+          <t>Programtext `Utveckling och lärande i förskoleklass och grundskolans åk 1–3` ≠ kursplanens namn `Utveckling och lärande i förskoleklass och grundskolans åk 1-3 (varav 7,5 hp VFU)` (kurskod `GPG3CF`); rad: - [[GPG3CF|Utveckling och lärande i förskoleklass och grundskolans åk 1–3]], 15 hp</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>L7I9A</t>
+          <t>LBF3A</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1346,24 +1346,24 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>`Sociala relationer, konflikter och makt för ämneslärare årskurs 7–9 - AIL` (7,5 hp); rad: - Sociala relationer, konflikter och makt för ämneslärare årskurs 7–9 - AIL, 7,5 hp</t>
+          <t>Programtext `Sociala relationer, konflikter och makt i förskoleklass och grundskolan åk 1–3` ≠ kursplanens namn `Sociala relationer, konflikter och makt i förskoleklass och grundskolan åk 1-3 (varav 7,5 hp VFU)` (kurskod `GPG2M9`); rad: - [[GPG2M9|Sociala relationer, konflikter och makt i förskoleklass och grundskolan åk 1–3]], 15 hp</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=L7I9A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>L7I9A</t>
+          <t>LBF3A</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1373,24 +1373,24 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>`Utvärdering och utvecklingsarbete för ämneslärare årskurs 7–9 – AIL` (7,5 hp); rad: - Utvärdering och utvecklingsarbete för ämneslärare årskurs 7–9 – AIL, 7,5 hp</t>
+          <t>Programtext `Vetenskapsteori och utbildningsvetenskaplig forskning för grundlärare F -3` ≠ kursplanens namn `Vetenskapsteori och utbildningsvetenskaplig forskning för grundlärare F-3` (kurskod `APG244`); rad: - [[APG244|Vetenskapsteori och utbildningsvetenskaplig forskning för grundlärare F -3]], 7,5 hp</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=L7I9A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>L7I9A</t>
+          <t>LBF3A</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1400,24 +1400,24 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>`Verksamhetsförlagd utbildning 3 för ämneslärare årskurs 7–9 - AIL` (15 hp); rad: - Verksamhetsförlagd utbildning 3 för ämneslärare årskurs 7–9 - AIL, 15 hp</t>
+          <t>Programtext `Engelska för grundlärare åk F-3` ≠ kursplanens namn `Engelska för grundlärare F-3` (kurskod `GEN2BJ`); rad: - &lt;a class="no-graph" href="GEN2BJ"&gt;Engelska för grundlärare åk F-3&lt;/a&gt;, 15 hp</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=L7I9A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>L7I9A</t>
+          <t>LP79A</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1432,19 +1432,19 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>`Vetenskapsteori och utbildningsvetenskaplig forskning för ämneslärare årskurs 7–9 - AIL` (7,5 hp); rad: - Vetenskapsteori och utbildningsvetenskaplig forskning för ämneslärare årskurs 7–9 - AIL, 7,5 hp</t>
+          <t>`Utveckling och lärande - ämneslärare` (15 hp); rad: - Utveckling och lärande - ämneslärare, 15 hp</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=L7I9A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LP79A</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>L7I9A</t>
+          <t>LP79A</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1459,19 +1459,19 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>`_Examensarbete i matematik för ämneslärarexamen inriktning grundskolans årskurs 7–9` (15 hp); rad: - _Examensarbete i matematik för ämneslärarexamen inriktning grundskolans årskurs 7–9, 15 hp</t>
+          <t>`Utveckling och lärande för ämneslärare inriktning åk 7-9` (15 hp); rad: - Utveckling och lärande för ämneslärare inriktning åk 7-9, 15 hp</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=L7I9A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LP79A</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>LBF3A</t>
+          <t>LP79A</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1486,19 +1486,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>`Didaktik och ledarskap i förskoleklass och grundskolans åk 1–3` (15 hp); rad: - Didaktik och ledarskap i förskoleklass och grundskolans åk 1–3, 15 hp</t>
+          <t>`Sociala relationer, konflikter och makt - ämneslärare` (7,5 hp); rad: - Sociala relationer, konflikter och makt - ämneslärare, 7,5 hp</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LP79A</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>LBF3A</t>
+          <t>LP79A</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1513,19 +1513,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>`Utvärdering och utvecklingsarbete i förskoleklass och grundskolans åk 1–3` (15 hp); rad: - Utvärdering och utvecklingsarbete i förskoleklass och grundskolans åk 1–3, 15 hp</t>
+          <t>`Utvärdering och utvecklingsarbete för ämneslärare` (7,5 hp); rad: - Utvärdering och utvecklingsarbete för ämneslärare, 7,5 hp</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LP79A</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>LBF3A</t>
+          <t>LP79A</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1535,24 +1535,24 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Programtext `Utveckling och lärande i förskoleklass och grundskolans åk 1–3` ≠ kursplanens namn `Utveckling och lärande i förskoleklass och grundskolans åk 1-3 (varav 7,5 hp VFU)` (kurskod `GPG3CF`); rad: - [[GPG3CF|Utveckling och lärande i förskoleklass och grundskolans åk 1–3]], 15 hp</t>
+          <t>`Verksamhetsförlagd utbildning - ämneslärare` (15 hp); rad: - Verksamhetsförlagd utbildning - ämneslärare, 15 hp</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LP79A</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>LBF3A</t>
+          <t>LPGYA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1562,24 +1562,24 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Programtext `Sociala relationer, konflikter och makt i förskoleklass och grundskolan åk 1–3` ≠ kursplanens namn `Sociala relationer, konflikter och makt i förskoleklass och grundskolan åk 1-3 (varav 7,5 hp VFU)` (kurskod `GPG2M9`); rad: - [[GPG2M9|Sociala relationer, konflikter och makt i förskoleklass och grundskolan åk 1–3]], 15 hp</t>
+          <t>`Didaktik och ledarskap för ämneslärare inriktning gymnasieskolan` (15 hp); rad: - Didaktik och ledarskap för ämneslärare inriktning gymnasieskolan, 15 hp</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LPGYA</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>LBF3A</t>
+          <t>LPGYA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1589,24 +1589,24 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Programtext `Vetenskapsteori och utbildningsvetenskaplig forskning för grundlärare F -3` ≠ kursplanens namn `Vetenskapsteori och utbildningsvetenskaplig forskning för grundlärare F-3` (kurskod `APG244`); rad: - [[APG244|Vetenskapsteori och utbildningsvetenskaplig forskning för grundlärare F -3]], 7,5 hp</t>
+          <t>`Utveckling och lärande - ämneslärare` (15 hp); rad: - Utveckling och lärande - ämneslärare, 15 hp</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LPGYA</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>LBF3A</t>
+          <t>LPGYA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1616,24 +1616,24 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Programtext `Svenska 1 för grundlärare F-3: Barns språkutveckling, språklig variation samt barn- och ungdomslitteratur` ≠ kursplanens namn `Svenska 1 för grundlärare F-3` (kurskod `GSV2ZV`); rad: - &lt;a class="no-graph" href="GSV2ZV"&gt;Svenska 1 för grundlärare F-3: Barns språkutveckling, språklig variation samt barn- och ungdomslitteratur&lt;/a&gt;, 15 hp</t>
+          <t>`Sociala relationer, konflikter och makt - ämneslärare` (7,5 hp); rad: - Sociala relationer, konflikter och makt - ämneslärare, 7,5 hp</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LPGYA</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>LBF3A</t>
+          <t>LPGYA</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1643,24 +1643,24 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Programtext `Engelska för grundlärare åk F-3` ≠ kursplanens namn `Engelska för grundlärare F-3` (kurskod `GEN2BJ`); rad: - &lt;a class="no-graph" href="GEN2BJ"&gt;Engelska för grundlärare åk F-3&lt;/a&gt;, 15 hp</t>
+          <t>`Utvärdering och utvecklingsarbete för ämneslärare` (7,5 hp); rad: - Utvärdering och utvecklingsarbete för ämneslärare, 7,5 hp</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LPGYA</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>LBF3A</t>
+          <t>LPGYA</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1670,24 +1670,24 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Programtext `Svenska 2 för grundlärare F-3: Läs- och skrivutveckling och läs- och skrivundervisning` ≠ kursplanens namn `Svenska 2 för grundlärare F-3` (kurskod `GSV2ZW`); rad: - &lt;a class="no-graph" href="GSV2ZW"&gt;Svenska 2 för grundlärare F-3: Läs- och skrivutveckling och läs- och skrivundervisning&lt;/a&gt;, 15 hp</t>
+          <t>`Verksamhetsförlagd utbildning - ämneslärare` (15 hp); rad: - Verksamhetsförlagd utbildning - ämneslärare, 15 hp</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LBF3A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LPGYA</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>LP79A</t>
+          <t>LVALA</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1697,24 +1697,24 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>`Utveckling och lärande - ämneslärare` (15 hp); rad: - Utveckling och lärande - ämneslärare, 15 hp</t>
+          <t>Programtext `Skolans samhällsuppdrag` ≠ kursplanens namn `Skolans samhällsuppdrag - VAL` (kurskod `GPG2Z7`); rad: - [[GPG2Z7|Skolans samhällsuppdrag]], 7,5 hp</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LP79A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>LP79A</t>
+          <t>LVALA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1724,24 +1724,24 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>`Utveckling och lärande för ämneslärare inriktning åk 7-9` (15 hp); rad: - Utveckling och lärande för ämneslärare inriktning åk 7-9, 15 hp</t>
+          <t>Programtext `Didaktik och ledarskap` ≠ kursplanens namn `Didaktik och ledarskap - VAL` (kurskod `GPG3BE`); rad: - [[GPG3BE|Didaktik och ledarskap]], 7,5 hp</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LP79A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>LP79A</t>
+          <t>LVALA</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1751,24 +1751,24 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>`Sociala relationer, konflikter och makt - ämneslärare` (7,5 hp); rad: - Sociala relationer, konflikter och makt - ämneslärare, 7,5 hp</t>
+          <t>Programtext `Utveckling och lärande` ≠ kursplanens namn `Utveckling och lärande - VAL` (kurskod `GPG2Z4`); rad: - [[GPG2Z4|Utveckling och lärande]], 7,5 hp</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LP79A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>LP79A</t>
+          <t>LVALA</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1778,24 +1778,24 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>`Utvärdering och utvecklingsarbete för ämneslärare` (7,5 hp); rad: - Utvärdering och utvecklingsarbete för ämneslärare, 7,5 hp</t>
+          <t>Programtext `Sociala relationer och konflikthantering` ≠ kursplanens namn `Sociala relationer och konflikthantering - VAL` (kurskod `GPG2Z6`); rad: - [[GPG2Z6|Sociala relationer och konflikthantering]], 7,5 hp</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LP79A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>LP79A</t>
+          <t>LVALA</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1805,24 +1805,24 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>`Verksamhetsförlagd utbildning - ämneslärare` (15 hp); rad: - Verksamhetsförlagd utbildning - ämneslärare, 15 hp</t>
+          <t>Programtext `Vetenskapsteori och utbildningsvetenskaplig forskning` ≠ kursplanens namn `Vetenskapsteori och utbildningsvetenskaplig forskning - VAL` (kurskod `APG28M`); rad: - [[APG28M|Vetenskapsteori och utbildningsvetenskaplig forskning]], 7,5 hp</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LP79A</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>LPGYA</t>
+          <t>LVALA</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1832,24 +1832,24 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>`Didaktik och ledarskap för ämneslärare inriktning gymnasieskolan` (15 hp); rad: - Didaktik och ledarskap för ämneslärare inriktning gymnasieskolan, 15 hp</t>
+          <t>Programtext `Utvärdering och utvecklingsarbete` ≠ kursplanens namn `Utvärdering och utvecklingsarbete - VAL` (kurskod `GPG3FU`); rad: - [[GPG3FU|Utvärdering och utvecklingsarbete]], 7,5 hp</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LPGYA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>LPGYA</t>
+          <t>LVALA</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1859,24 +1859,24 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>`Utveckling och lärande - ämneslärare` (15 hp); rad: - Utveckling och lärande - ämneslärare, 15 hp</t>
+          <t>Programtext `Självständigt arbete` ≠ kursplanens namn `Självständigt arbete - VAL` (kurskod `GPG3FV`); rad: - [[GPG3FV|Självständigt arbete]], 7,5 hp</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LPGYA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>LPGYA</t>
+          <t>LVALA</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1886,24 +1886,24 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>`Sociala relationer, konflikter och makt - ämneslärare` (7,5 hp); rad: - Sociala relationer, konflikter och makt - ämneslärare, 7,5 hp</t>
+          <t>Programtext `Verksamhetsförlagd utbildning 1` ≠ kursplanens namn `Verksamhetsförlagd utbildning 1 - VAL` (kurskod `GPG3FS`); rad: - [[GPG3FS|Verksamhetsförlagd utbildning 1]], 7,5 hp</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LPGYA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>LPGYA</t>
+          <t>LVALA</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1913,24 +1913,24 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>`Utvärdering och utvecklingsarbete för ämneslärare` (7,5 hp); rad: - Utvärdering och utvecklingsarbete för ämneslärare, 7,5 hp</t>
+          <t>Programtext `Verksamhetsförlagd utbildning 2` ≠ kursplanens namn `Verksamhetsförlagd utbildning 2 - VAL` (kurskod `GPG3FT`); rad: - [[GPG3FT|Verksamhetsförlagd utbildning 2]], 15 hp</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LPGYA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>LPGYA</t>
+          <t>LVALA</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1940,17 +1940,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>`Verksamhetsförlagd utbildning - ämneslärare` (15 hp); rad: - Verksamhetsförlagd utbildning - ämneslärare, 15 hp</t>
+          <t>Programtext `Verksamhetsförlagd utbildning 3` ≠ kursplanens namn `Verksamhetsförlagd utbildning 3 - VAL` (kurskod `APG2BK`); rad: - [[APG2BK|Verksamhetsförlagd utbildning 3]], 7,5 hp</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LPGYA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Programtext `Skolans samhällsuppdrag` ≠ kursplanens namn `Skolans samhällsuppdrag - VAL` (kurskod `GPG2Z7`); rad: - [[GPG2Z7|Skolans samhällsuppdrag]], 7,5 hp</t>
+          <t>Programtext `Didaktik och bedömning` ≠ kursplanens namn `Didaktik och bedömning - VAL` (kurskod `GPG33F`); rad: - [[GPG33F|Didaktik och bedömning]], 7,5 hp</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Programtext `Didaktik och ledarskap` ≠ kursplanens namn `Didaktik och ledarskap - VAL` (kurskod `GPG3BE`); rad: - [[GPG3BE|Didaktik och ledarskap]], 7,5 hp</t>
+          <t>Programtext `Utveckling, lärande och ledarskap` ≠ kursplanens namn `Utveckling, lärande och ledarskap - VAL` (kurskod `GPG33D`); rad: - [[GPG33D|Utveckling, lärande och ledarskap]], 7,5 hp</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Programtext `Utveckling och lärande` ≠ kursplanens namn `Utveckling och lärande - VAL` (kurskod `GPG2Z4`); rad: - [[GPG2Z4|Utveckling och lärande]], 7,5 hp</t>
+          <t>Programtext `Sociala relationer, skolans historiska utveckling och samhällsuppdrag` ≠ kursplanens namn `Sociala relationer, skolans historiska utveckling och samhällsuppdrag - VAL` (kurskod `GPG33E`); rad: - [[GPG33E|Sociala relationer, skolans historiska utveckling och samhällsuppdrag]], 7,5 hp</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -2038,7 +2038,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>LVALA</t>
+          <t>SBMPG</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2048,24 +2048,24 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Programtext `Sociala relationer och konflikthantering` ≠ kursplanens namn `Sociala relationer och konflikthantering - VAL` (kurskod `GPG2Z6`); rad: - [[GPG2Z6|Sociala relationer och konflikthantering]], 7,5 hp</t>
+          <t>`Makroekonomi introduktion` (7,5 hp); rad: - Makroekonomi introduktion, 7,5 hp</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SBMPG</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>LVALA</t>
+          <t>SBMPG</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2075,24 +2075,24 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Programtext `Vetenskapsteori och utbildningsvetenskaplig forskning` ≠ kursplanens namn `Vetenskapsteori och utbildningsvetenskaplig forskning - VAL` (kurskod `APG28M`); rad: - [[APG28M|Vetenskapsteori och utbildningsvetenskaplig forskning]], 7,5 hp</t>
+          <t>`Mikroekonomi introduktion` (7,5 hp); rad: - Mikroekonomi introduktion, 7,5 hp</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SBMPG</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>LVALA</t>
+          <t>SDUVA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2102,24 +2102,24 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Programtext `Utvärdering och utvecklingsarbete` ≠ kursplanens namn `Utvärdering och utvecklingsarbete - VAL` (kurskod `GPG3FU`); rad: - [[GPG3FU|Utvärdering och utvecklingsarbete]], 7,5 hp</t>
+          <t>`Evenemangsturism` (7,5 hp); rad: - Evenemangsturism, 7,5 hp</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SDUVA</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>LVALA</t>
+          <t>SENGR</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2129,24 +2129,24 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Programtext `Självständigt arbete` ≠ kursplanens namn `Självständigt arbete - VAL` (kurskod `GPG3FV`); rad: - [[GPG3FV|Självständigt arbete]], 7,5 hp</t>
+          <t>`Makroekonomi introduktion` (7,5 hp); rad: - Makroekonomi introduktion, 7,5 hp</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SENGR</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>LVALA</t>
+          <t>SENGR</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2156,24 +2156,24 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Programtext `Verksamhetsförlagd utbildning 1` ≠ kursplanens namn `Verksamhetsförlagd utbildning 1 - VAL` (kurskod `GPG3FS`); rad: - [[GPG3FS|Verksamhetsförlagd utbildning 1]], 7,5 hp</t>
+          <t>`Mikroekonomi introduktion` (7,5 hp); rad: - Mikroekonomi introduktion, 7,5 hp</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SENGR</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>LVALA</t>
+          <t>SENGR</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2183,24 +2183,24 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Programtext `Verksamhetsförlagd utbildning 2` ≠ kursplanens namn `Verksamhetsförlagd utbildning 2 - VAL` (kurskod `GPG3FT`); rad: - [[GPG3FT|Verksamhetsförlagd utbildning 2]], 15 hp</t>
+          <t>`Mikroekonomi fortsättningskurs` (7,5 hp); rad: - Mikroekonomi fortsättningskurs, 7,5 hp</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SENGR</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>LVALA</t>
+          <t>SENGR</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2210,24 +2210,24 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Programtext `Verksamhetsförlagd utbildning 3` ≠ kursplanens namn `Verksamhetsförlagd utbildning 3 - VAL` (kurskod `APG2BK`); rad: - [[APG2BK|Verksamhetsförlagd utbildning 3]], 7,5 hp</t>
+          <t>`Makroekonomi fortsättning` (7,5 hp); rad: - Makroekonomi fortsättning, 7,5 hp</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SENGR</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>LVALA</t>
+          <t>SENGR</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2237,24 +2237,24 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Programtext `Didaktik och bedömning` ≠ kursplanens namn `Didaktik och bedömning - VAL` (kurskod `GPG33F`); rad: - [[GPG33F|Didaktik och bedömning]], 7,5 hp</t>
+          <t>`Samhällsekonomisk utvärdering av offentliga projekt` (7,5 hp); rad: - Samhällsekonomisk utvärdering av offentliga projekt, 7,5 hp</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SENGR</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>LVALA</t>
+          <t>SEPFG</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2264,24 +2264,24 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Programtext `Utveckling, lärande och ledarskap` ≠ kursplanens namn `Utveckling, lärande och ledarskap - VAL` (kurskod `GPG33D`); rad: - [[GPG33D|Utveckling, lärande och ledarskap]], 7,5 hp</t>
+          <t>`Entreprenörskap - entreprenörskapets villkor och särart` (7,5 hp); rad: - Entreprenörskap - entreprenörskapets villkor och särart, 7,5 hp</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SEPFG</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>LVALA</t>
+          <t>SEPFG</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2291,24 +2291,24 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Programtext `Sociala relationer, skolans historiska utveckling och samhällsuppdrag` ≠ kursplanens namn `Sociala relationer, skolans historiska utveckling och samhällsuppdrag - VAL` (kurskod `GPG33E`); rad: - [[GPG33E|Sociala relationer, skolans historiska utveckling och samhällsuppdrag]], 7,5 hp</t>
+          <t>`Förhandlings  försäljnings  och dialogkonst` (7,5 hp); rad: - Förhandlings  försäljnings  och dialogkonst, 7,5 hp</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SEPFG</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>SBMPG</t>
+          <t>SFIFA</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2323,19 +2323,19 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>`Makroekonomi introduktion` (7,5 hp); rad: - Makroekonomi introduktion, 7,5 hp</t>
+          <t>`Studier i Internationell Human Resource Management` (15 hp); rad: - Studier i Internationell Human Resource Management, 15 hp</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SBMPG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SFIFA</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>SBMPG</t>
+          <t>SMINA</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2350,19 +2350,19 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>`Mikroekonomi introduktion` (7,5 hp); rad: - Mikroekonomi introduktion, 7,5 hp</t>
+          <t>`Avancerad mikroteori` (7,5 hp); rad: - Avancerad mikroteori, 7,5 hp</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SBMPG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SMINA</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>SDUVA</t>
+          <t>SMINA</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2377,19 +2377,19 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>`Evenemangsturism` (7,5 hp); rad: - Evenemangsturism, 7,5 hp</t>
+          <t>`Samhällsekonomisk utvärdering av offentliga projekt` (7,5 hp); rad: - Samhällsekonomisk utvärdering av offentliga projekt, 7,5 hp</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SDUVA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SMINA</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>SENGR</t>
+          <t>SPARG</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2404,19 +2404,19 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>`Makroekonomi introduktion` (7,5 hp); rad: - Makroekonomi introduktion, 7,5 hp</t>
+          <t>`Arbetsrätt i personalarbetets praktik` (15 hp); rad: - Arbetsrätt i personalarbetets praktik, 15 hp</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SENGR</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>SENGR</t>
+          <t>SPARG</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2431,19 +2431,19 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>`Mikroekonomi introduktion` (7,5 hp); rad: - Mikroekonomi introduktion, 7,5 hp</t>
+          <t>`Grunder i personalekonomisk styrning` (15 hp); rad: - Grunder i personalekonomisk styrning, 15 hp</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SENGR</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>SENGR</t>
+          <t>SPARG</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2458,19 +2458,19 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>`Mikroekonomi fortsättningskurs` (7,5 hp); rad: - Mikroekonomi fortsättningskurs, 7,5 hp</t>
+          <t>`Personalarbete med praktik` (15 hp); rad: - Personalarbete med praktik, 15 hp</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SENGR</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>SENGR</t>
+          <t>SPARG</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2485,19 +2485,19 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>`Makroekonomi fortsättning` (7,5 hp); rad: - Makroekonomi fortsättning, 7,5 hp</t>
+          <t>`Arbetsmarknad i ett jämförande internationellt perspektiv` (7,5 hp); rad: - Arbetsmarknad i ett jämförande internationellt perspektiv, 7,5 hp</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SENGR</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>SENGR</t>
+          <t>SPARG</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2512,19 +2512,19 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>`Samhällsekonomisk utvärdering av offentliga projekt` (7,5 hp); rad: - Samhällsekonomisk utvärdering av offentliga projekt, 7,5 hp</t>
+          <t>`Arbetsmiljökunskap i ett jämförande internationellt perspektiv` (7,5 hp); rad: - Arbetsmiljökunskap i ett jämförande internationellt perspektiv, 7,5 hp</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SENGR</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>SEPFG</t>
+          <t>SPARG</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2539,19 +2539,19 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>`Entreprenörskap - entreprenörskapets villkor och särart` (7,5 hp); rad: - Entreprenörskap - entreprenörskapets villkor och särart, 7,5 hp</t>
+          <t>`Examensarbete inom arbetsvetenskap` (15 hp); rad: - Examensarbete inom arbetsvetenskap, 15 hp</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SEPFG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>SEPFG</t>
+          <t>SPARG</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2566,19 +2566,19 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>`Förhandlings  försäljnings  och dialogkonst` (7,5 hp); rad: - Förhandlings  försäljnings  och dialogkonst, 7,5 hp</t>
+          <t>`Forskningsprocess och analysmetoder` (7,5 hp); rad: - Forskningsprocess och analysmetoder, 7,5 hp</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SEPFG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>SFIFA</t>
+          <t>SPARG</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2593,19 +2593,19 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>`Studier i Internationell Human Resource Management` (15 hp); rad: - Studier i Internationell Human Resource Management, 15 hp</t>
+          <t>`Komplexa arbetsorganisationer` (7,5 hp); rad: - Komplexa arbetsorganisationer, 7,5 hp</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SFIFA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>SFIFA</t>
+          <t>SPARG</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2615,24 +2615,24 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Programtext avviker från kursplanens namn</t>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Programtext `Examensarbete` ≠ kursplanens namn `Tyska: Examensarbete` (kurskod `TY2007`); rad: - &lt;a class="no-graph" href="TY2007"&gt;Examensarbete&lt;/a&gt;, 15 hp</t>
+          <t>`Komplexa sociala processer i arbetslivet` (7,5 hp); rad: - Komplexa sociala processer i arbetslivet, 7,5 hp</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SFIFA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>SMINA</t>
+          <t>SPARG</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2647,19 +2647,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>`Avancerad mikroteori` (7,5 hp); rad: - Avancerad mikroteori, 7,5 hp</t>
+          <t>`Vetenskap och metod` (7,5 hp); rad: - Vetenskap och metod, 7,5 hp</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SMINA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>SMINA</t>
+          <t>SSHVG</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2674,19 +2674,19 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>`Samhällsekonomisk utvärdering av offentliga projekt` (7,5 hp); rad: - Samhällsekonomisk utvärdering av offentliga projekt, 7,5 hp</t>
+          <t>`Inriktning sociologi II` (30 hp); rad: - Inriktning sociologi II, 30 hp</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SMINA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>SPARG</t>
+          <t>SSHVG</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2701,19 +2701,19 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>`Arbetsrätt i personalarbetets praktik` (15 hp); rad: - Arbetsrätt i personalarbetets praktik, 15 hp</t>
+          <t>`Examensarbete för högskoleexamen i Sociologi` (7,5 hp); rad: - Examensarbete för högskoleexamen i Sociologi, 7,5 hp</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>SPARG</t>
+          <t>SSHVG</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2728,19 +2728,19 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>`Grunder i personalekonomisk styrning` (15 hp); rad: - Grunder i personalekonomisk styrning, 15 hp</t>
+          <t>`Makt och samhälle` (7,5 hp); rad: - Makt och samhälle, 7,5 hp</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>SPARG</t>
+          <t>SSHVG</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2755,19 +2755,19 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>`Personalarbete med praktik` (15 hp); rad: - Personalarbete med praktik, 15 hp</t>
+          <t>`Samhällsvetenskapliga metoder I` (7,5 hp); rad: - Samhällsvetenskapliga metoder I, 7,5 hp</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>SPARG</t>
+          <t>SSHVG</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2782,19 +2782,19 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>`Arbetsmarknad i ett jämförande internationellt perspektiv` (7,5 hp); rad: - Arbetsmarknad i ett jämförande internationellt perspektiv, 7,5 hp</t>
+          <t>`Inriktning statsvetenskap II` (30 hp); rad: - Inriktning statsvetenskap II, 30 hp</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>SPARG</t>
+          <t>SSHVG</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2809,19 +2809,19 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>`Arbetsmiljökunskap i ett jämförande internationellt perspektiv` (7,5 hp); rad: - Arbetsmiljökunskap i ett jämförande internationellt perspektiv, 7,5 hp</t>
+          <t>`Inriktning sociologi III` (30 hp); rad: - Inriktning sociologi III, 30 hp</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>SPARG</t>
+          <t>SSHVG</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2836,19 +2836,19 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>`Examensarbete inom arbetsvetenskap` (15 hp); rad: - Examensarbete inom arbetsvetenskap, 15 hp</t>
+          <t>`Examensarbete för kandidatexamen i sociologi` (15 hp); rad: - Examensarbete för kandidatexamen i sociologi, 15 hp</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>SPARG</t>
+          <t>SSHVG</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2863,19 +2863,19 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>`Forskningsprocess och analysmetoder` (7,5 hp); rad: - Forskningsprocess och analysmetoder, 7,5 hp</t>
+          <t>`Fördjupningskurs i sociologisk teori` (7,5 hp); rad: - Fördjupningskurs i sociologisk teori, 7,5 hp</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>SPARG</t>
+          <t>SSHVG</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2890,19 +2890,19 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>`Komplexa arbetsorganisationer` (7,5 hp); rad: - Komplexa arbetsorganisationer, 7,5 hp</t>
+          <t>`Samhällsvetenskapliga metoder II` (7,5 hp); rad: - Samhällsvetenskapliga metoder II, 7,5 hp</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>SPARG</t>
+          <t>SSHVG</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2917,19 +2917,19 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>`Komplexa sociala processer i arbetslivet` (7,5 hp); rad: - Komplexa sociala processer i arbetslivet, 7,5 hp</t>
+          <t>`Inriktning statsvetenskap III` (30 hp); rad: - Inriktning statsvetenskap III, 30 hp</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>SPARG</t>
+          <t>SSHVG</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2944,12 +2944,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>`Vetenskap och metod` (7,5 hp); rad: - Vetenskap och metod, 7,5 hp</t>
+          <t>`Samhällsvetenskapliga metoder II inriktning statsvetenskap` (7,5 hp); rad: - Samhällsvetenskapliga metoder II inriktning statsvetenskap, 7,5 hp</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
         </is>
       </c>
     </row>
@@ -2966,12 +2966,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Kursraden ser avbruten/feltrycklig ut</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>`Inriktning sociologi II` (30 hp); rad: - Inriktning sociologi II, 30 hp</t>
+          <t>`Valbar termin (med möjlighet till internationellt utbyte eller läsning av valfri temakurs/kurser om` (30 hp); rad: - Valbar termin (med möjlighet till internationellt utbyte eller läsning av valfri temakurs/kurser om, 30 hp</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2983,7 +2983,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>SSHVG</t>
+          <t>STMGG</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2998,19 +2998,19 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>`Examensarbete för högskoleexamen i Sociologi` (7,5 hp); rad: - Examensarbete för högskoleexamen i Sociologi, 7,5 hp</t>
+          <t>`Festival och Event Management` (7,5 hp); rad: - Festival och Event Management, 7,5 hp</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=STMGG</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>SSHVG</t>
+          <t>STMGG</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3025,19 +3025,19 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>`Makt och samhälle` (7,5 hp); rad: - Makt och samhälle, 7,5 hp</t>
+          <t>`Turismstudier utomlands` (30 hp); rad: - Turismstudier utomlands, 30 hp</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=STMGG</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>SSHVG</t>
+          <t>STMGG</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3052,314 +3052,17 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>`Samhällsvetenskapliga metoder I` (7,5 hp); rad: - Samhällsvetenskapliga metoder I, 7,5 hp</t>
+          <t>`Kvantitativa forskningsmetoder` (7,5 hp); rad: - Kvantitativa forskningsmetoder, 7,5 hp</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>SSHVG</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>`Inriktning statsvetenskap II` (30 hp); rad: - Inriktning statsvetenskap II, 30 hp</t>
-        </is>
-      </c>
-      <c r="E98" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="2" t="inlineStr">
-        <is>
-          <t>SSHVG</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>`Inriktning sociologi III` (30 hp); rad: - Inriktning sociologi III, 30 hp</t>
-        </is>
-      </c>
-      <c r="E99" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>SSHVG</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>`Examensarbete för kandidatexamen i sociologi` (15 hp); rad: - Examensarbete för kandidatexamen i sociologi, 15 hp</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="2" t="inlineStr">
-        <is>
-          <t>SSHVG</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>`Fördjupningskurs i sociologisk teori` (7,5 hp); rad: - Fördjupningskurs i sociologisk teori, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>SSHVG</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>`Samhällsvetenskapliga metoder II` (7,5 hp); rad: - Samhällsvetenskapliga metoder II, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>SSHVG</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>`Inriktning statsvetenskap III` (30 hp); rad: - Inriktning statsvetenskap III, 30 hp</t>
-        </is>
-      </c>
-      <c r="E103" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>SSHVG</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>`Samhällsvetenskapliga metoder II inriktning statsvetenskap` (7,5 hp); rad: - Samhällsvetenskapliga metoder II inriktning statsvetenskap, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="2" t="inlineStr">
-        <is>
-          <t>SSHVG</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>Kursraden ser avbruten/feltrycklig ut</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>`Valbar termin (med möjlighet till internationellt utbyte eller läsning av valfri temakurs/kurser om` (30 hp); rad: - Valbar termin (med möjlighet till internationellt utbyte eller läsning av valfri temakurs/kurser om, 30 hp</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>STMGG</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>`Festival och Event Management` (7,5 hp); rad: - Festival och Event Management, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=STMGG</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>STMGG</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>`Turismstudier utomlands` (30 hp); rad: - Turismstudier utomlands, 30 hp</t>
-        </is>
-      </c>
-      <c r="E107" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=STMGG</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>STMGG</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>`Kvantitativa forskningsmetoder` (7,5 hp); rad: - Kvantitativa forskningsmetoder, 7,5 hp</t>
-        </is>
-      </c>
-      <c r="E108" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=STMGG</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E108"/>
+  <autoFilter ref="A1:E97"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -3553,28 +3256,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="rId190"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A97" r:id="rId191"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A98" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A99" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A100" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A101" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A102" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E102" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A103" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A104" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A105" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A106" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A107" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A108" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="rId214"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>